<commit_message>
feat: updated student import script and template with 11 new students
</commit_message>
<xml_diff>
--- a/server/scripts/students-template-2.xlsx
+++ b/server/scripts/students-template-2.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\vinee\Desktop\AG Projects\school-management\server\scripts\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{626C737A-FA96-4E5A-9306-67096A67FA10}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FC661C69-9387-402C-9D71-607FE24073BE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="325" uniqueCount="92">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="424" uniqueCount="114">
   <si>
     <t>admissionNo</t>
   </si>
@@ -301,6 +301,72 @@
   </si>
   <si>
     <t>Abdul Hakeem Cheriyan Parambil</t>
+  </si>
+  <si>
+    <t>Anviya MV</t>
+  </si>
+  <si>
+    <t>Vipin M</t>
+  </si>
+  <si>
+    <t>Shahla Fathima</t>
+  </si>
+  <si>
+    <t>Muhammed Shafi</t>
+  </si>
+  <si>
+    <t>Muhammed Sinan UT</t>
+  </si>
+  <si>
+    <t>Abdul Hakeem UT</t>
+  </si>
+  <si>
+    <t>Fathima Sidra</t>
+  </si>
+  <si>
+    <t>Ajwa Mariyam K</t>
+  </si>
+  <si>
+    <t>Unais MV</t>
+  </si>
+  <si>
+    <t>Musthafa KK</t>
+  </si>
+  <si>
+    <t>Bijoy Bhaskaran M</t>
+  </si>
+  <si>
+    <t>Nafsal A</t>
+  </si>
+  <si>
+    <t>Adam Nafsal A</t>
+  </si>
+  <si>
+    <t>Sreehan Vineeth</t>
+  </si>
+  <si>
+    <t>Vineeth MP</t>
+  </si>
+  <si>
+    <t>Muhammad hanan KV</t>
+  </si>
+  <si>
+    <t>Sudheer</t>
+  </si>
+  <si>
+    <t>Shazia Sajid</t>
+  </si>
+  <si>
+    <t>Adhilakshmi Bijoy</t>
+  </si>
+  <si>
+    <t>Sajid Muhammed</t>
+  </si>
+  <si>
+    <t>Nihaya Binth Ahammed VK</t>
+  </si>
+  <si>
+    <t>Nisar Ahammed VK</t>
   </si>
 </sst>
 </file>
@@ -619,7 +685,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:Q47"/>
+  <dimension ref="A1:Q59"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="11.109375" customWidth="1"/>
@@ -2162,6 +2228,490 @@
         <v>22</v>
       </c>
     </row>
+    <row r="49" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A49">
+        <v>2526</v>
+      </c>
+      <c r="B49" s="1">
+        <v>45798</v>
+      </c>
+      <c r="C49">
+        <v>1026</v>
+      </c>
+      <c r="D49" t="s">
+        <v>92</v>
+      </c>
+      <c r="E49" t="s">
+        <v>21</v>
+      </c>
+      <c r="F49" t="s">
+        <v>17</v>
+      </c>
+      <c r="H49" t="s">
+        <v>18</v>
+      </c>
+      <c r="I49" s="1">
+        <v>44041</v>
+      </c>
+      <c r="J49" t="s">
+        <v>93</v>
+      </c>
+      <c r="K49">
+        <v>9946658562</v>
+      </c>
+      <c r="M49" t="s">
+        <v>20</v>
+      </c>
+      <c r="N49" t="s">
+        <v>51</v>
+      </c>
+      <c r="O49" t="s">
+        <v>17</v>
+      </c>
+      <c r="P49" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="50" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A50">
+        <v>2551</v>
+      </c>
+      <c r="B50" s="1">
+        <v>45810</v>
+      </c>
+      <c r="C50">
+        <v>1051</v>
+      </c>
+      <c r="D50" t="s">
+        <v>94</v>
+      </c>
+      <c r="E50" t="s">
+        <v>21</v>
+      </c>
+      <c r="F50" t="s">
+        <v>17</v>
+      </c>
+      <c r="H50" t="s">
+        <v>18</v>
+      </c>
+      <c r="I50" s="1">
+        <v>43702</v>
+      </c>
+      <c r="J50" t="s">
+        <v>95</v>
+      </c>
+      <c r="K50">
+        <v>9048606725</v>
+      </c>
+      <c r="M50" t="s">
+        <v>20</v>
+      </c>
+      <c r="N50" t="s">
+        <v>51</v>
+      </c>
+      <c r="O50" t="s">
+        <v>17</v>
+      </c>
+      <c r="P50" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="51" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A51">
+        <v>2550</v>
+      </c>
+      <c r="B51" s="1">
+        <v>45810</v>
+      </c>
+      <c r="C51">
+        <v>1050</v>
+      </c>
+      <c r="D51" t="s">
+        <v>96</v>
+      </c>
+      <c r="E51" t="s">
+        <v>21</v>
+      </c>
+      <c r="F51" t="s">
+        <v>17</v>
+      </c>
+      <c r="H51" t="s">
+        <v>27</v>
+      </c>
+      <c r="I51" s="1">
+        <v>43771</v>
+      </c>
+      <c r="J51" t="s">
+        <v>97</v>
+      </c>
+      <c r="K51">
+        <v>9605416350</v>
+      </c>
+      <c r="M51" t="s">
+        <v>20</v>
+      </c>
+      <c r="N51" t="s">
+        <v>51</v>
+      </c>
+      <c r="O51" t="s">
+        <v>17</v>
+      </c>
+      <c r="P51" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="52" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A52">
+        <v>2554</v>
+      </c>
+      <c r="B52" s="1">
+        <v>45810</v>
+      </c>
+      <c r="C52">
+        <v>1054</v>
+      </c>
+      <c r="D52" t="s">
+        <v>98</v>
+      </c>
+      <c r="E52" t="s">
+        <v>21</v>
+      </c>
+      <c r="F52" t="s">
+        <v>17</v>
+      </c>
+      <c r="H52" t="s">
+        <v>18</v>
+      </c>
+      <c r="I52" s="1">
+        <v>43778</v>
+      </c>
+      <c r="J52" t="s">
+        <v>100</v>
+      </c>
+      <c r="K52">
+        <v>8590691668</v>
+      </c>
+      <c r="M52" t="s">
+        <v>20</v>
+      </c>
+      <c r="N52" t="s">
+        <v>51</v>
+      </c>
+      <c r="O52" t="s">
+        <v>17</v>
+      </c>
+      <c r="P52" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="53" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A53">
+        <v>2559</v>
+      </c>
+      <c r="B53" s="1">
+        <v>45819</v>
+      </c>
+      <c r="C53">
+        <v>1059</v>
+      </c>
+      <c r="D53" t="s">
+        <v>99</v>
+      </c>
+      <c r="E53" t="s">
+        <v>21</v>
+      </c>
+      <c r="F53" t="s">
+        <v>17</v>
+      </c>
+      <c r="H53" t="s">
+        <v>18</v>
+      </c>
+      <c r="I53" s="1">
+        <v>43633</v>
+      </c>
+      <c r="J53" t="s">
+        <v>101</v>
+      </c>
+      <c r="K53">
+        <v>9562992652</v>
+      </c>
+      <c r="M53" t="s">
+        <v>20</v>
+      </c>
+      <c r="N53" t="s">
+        <v>51</v>
+      </c>
+      <c r="O53" t="s">
+        <v>17</v>
+      </c>
+      <c r="P53" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="54" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A54">
+        <v>2552</v>
+      </c>
+      <c r="B54" s="1">
+        <v>45810</v>
+      </c>
+      <c r="C54">
+        <v>1052</v>
+      </c>
+      <c r="D54" t="s">
+        <v>110</v>
+      </c>
+      <c r="E54" t="s">
+        <v>21</v>
+      </c>
+      <c r="F54" t="s">
+        <v>17</v>
+      </c>
+      <c r="H54" t="s">
+        <v>18</v>
+      </c>
+      <c r="I54" s="1">
+        <v>43553</v>
+      </c>
+      <c r="J54" t="s">
+        <v>102</v>
+      </c>
+      <c r="K54">
+        <v>9961977420</v>
+      </c>
+      <c r="M54" t="s">
+        <v>20</v>
+      </c>
+      <c r="N54" t="s">
+        <v>51</v>
+      </c>
+      <c r="O54" t="s">
+        <v>17</v>
+      </c>
+      <c r="P54" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="55" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A55">
+        <v>2549</v>
+      </c>
+      <c r="B55" s="1">
+        <v>45810</v>
+      </c>
+      <c r="C55">
+        <v>1049</v>
+      </c>
+      <c r="D55" t="s">
+        <v>104</v>
+      </c>
+      <c r="E55" t="s">
+        <v>21</v>
+      </c>
+      <c r="F55" t="s">
+        <v>17</v>
+      </c>
+      <c r="H55" t="s">
+        <v>18</v>
+      </c>
+      <c r="I55" s="1">
+        <v>43888</v>
+      </c>
+      <c r="J55" t="s">
+        <v>103</v>
+      </c>
+      <c r="K55">
+        <v>8590934180</v>
+      </c>
+      <c r="M55" t="s">
+        <v>20</v>
+      </c>
+      <c r="N55" t="s">
+        <v>51</v>
+      </c>
+      <c r="O55" t="s">
+        <v>17</v>
+      </c>
+      <c r="P55" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="56" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A56">
+        <v>2553</v>
+      </c>
+      <c r="B56" s="1">
+        <v>45810</v>
+      </c>
+      <c r="C56">
+        <v>1053</v>
+      </c>
+      <c r="D56" t="s">
+        <v>105</v>
+      </c>
+      <c r="E56" t="s">
+        <v>21</v>
+      </c>
+      <c r="F56" t="s">
+        <v>17</v>
+      </c>
+      <c r="H56" t="s">
+        <v>27</v>
+      </c>
+      <c r="I56" s="1">
+        <v>44061</v>
+      </c>
+      <c r="J56" t="s">
+        <v>106</v>
+      </c>
+      <c r="K56">
+        <v>9895830110</v>
+      </c>
+      <c r="M56" t="s">
+        <v>20</v>
+      </c>
+      <c r="N56" t="s">
+        <v>51</v>
+      </c>
+      <c r="O56" t="s">
+        <v>17</v>
+      </c>
+      <c r="P56" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="57" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A57">
+        <v>2546</v>
+      </c>
+      <c r="B57" s="1">
+        <v>45809</v>
+      </c>
+      <c r="C57">
+        <v>1046</v>
+      </c>
+      <c r="D57" t="s">
+        <v>107</v>
+      </c>
+      <c r="E57" t="s">
+        <v>21</v>
+      </c>
+      <c r="F57" t="s">
+        <v>17</v>
+      </c>
+      <c r="H57" t="s">
+        <v>27</v>
+      </c>
+      <c r="I57" s="1">
+        <v>43436</v>
+      </c>
+      <c r="J57" t="s">
+        <v>108</v>
+      </c>
+      <c r="K57">
+        <v>9562886878</v>
+      </c>
+      <c r="M57" t="s">
+        <v>20</v>
+      </c>
+      <c r="N57" t="s">
+        <v>51</v>
+      </c>
+      <c r="O57" t="s">
+        <v>17</v>
+      </c>
+      <c r="P57" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="58" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A58">
+        <v>2530</v>
+      </c>
+      <c r="B58" s="1">
+        <v>45810</v>
+      </c>
+      <c r="C58">
+        <v>1030</v>
+      </c>
+      <c r="D58" t="s">
+        <v>109</v>
+      </c>
+      <c r="E58" t="s">
+        <v>21</v>
+      </c>
+      <c r="F58" t="s">
+        <v>17</v>
+      </c>
+      <c r="H58" t="s">
+        <v>18</v>
+      </c>
+      <c r="I58" s="1">
+        <v>43575</v>
+      </c>
+      <c r="J58" t="s">
+        <v>111</v>
+      </c>
+      <c r="K58">
+        <v>9895212128</v>
+      </c>
+      <c r="M58" t="s">
+        <v>20</v>
+      </c>
+      <c r="N58" t="s">
+        <v>51</v>
+      </c>
+      <c r="O58" t="s">
+        <v>17</v>
+      </c>
+      <c r="P58" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="59" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A59">
+        <v>2503</v>
+      </c>
+      <c r="B59" s="1">
+        <v>45770</v>
+      </c>
+      <c r="C59">
+        <v>1003</v>
+      </c>
+      <c r="D59" t="s">
+        <v>112</v>
+      </c>
+      <c r="E59" t="s">
+        <v>21</v>
+      </c>
+      <c r="F59" t="s">
+        <v>17</v>
+      </c>
+      <c r="H59" t="s">
+        <v>18</v>
+      </c>
+      <c r="I59" s="1">
+        <v>43901</v>
+      </c>
+      <c r="J59" t="s">
+        <v>113</v>
+      </c>
+      <c r="K59">
+        <v>9633338888</v>
+      </c>
+      <c r="M59" t="s">
+        <v>20</v>
+      </c>
+      <c r="N59" t="s">
+        <v>51</v>
+      </c>
+      <c r="O59" t="s">
+        <v>17</v>
+      </c>
+      <c r="P59" t="s">
+        <v>22</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Update student entry template with new records
</commit_message>
<xml_diff>
--- a/server/scripts/students-template-2.xlsx
+++ b/server/scripts/students-template-2.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\vinee\Desktop\AG Projects\school-management\server\scripts\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/28b6fd7089743951/Desktop/AG-Projects/school-management/server/scripts/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FC661C69-9387-402C-9D71-607FE24073BE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="83" documentId="13_ncr:1_{FC661C69-9387-402C-9D71-607FE24073BE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{83D385E0-CD4E-4D04-9CA4-E1681532864A}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="424" uniqueCount="114">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="505" uniqueCount="132">
   <si>
     <t>admissionNo</t>
   </si>
@@ -367,6 +367,60 @@
   </si>
   <si>
     <t>Nisar Ahammed VK</t>
+  </si>
+  <si>
+    <t>Sulaiha Zaya</t>
+  </si>
+  <si>
+    <t>Grade 4</t>
+  </si>
+  <si>
+    <t>Mohammed Zakir</t>
+  </si>
+  <si>
+    <t>Grade 3</t>
+  </si>
+  <si>
+    <t>Advika MV</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Radhwa naseer V</t>
+  </si>
+  <si>
+    <t>Naseer V</t>
+  </si>
+  <si>
+    <t>Muhammed Shayan KV</t>
+  </si>
+  <si>
+    <t>Abdul Muneer KV</t>
+  </si>
+  <si>
+    <t>Muhammed Zayan Anshif</t>
+  </si>
+  <si>
+    <t>Fasil KP</t>
+  </si>
+  <si>
+    <t>Fathima Zahra MV</t>
+  </si>
+  <si>
+    <t>Fathima Anshifa KV</t>
+  </si>
+  <si>
+    <t>Abdul Jaleel</t>
+  </si>
+  <si>
+    <t>Muhammed Aznan P</t>
+  </si>
+  <si>
+    <t>Shaji P</t>
+  </si>
+  <si>
+    <t>Naeem Muhammed KH</t>
+  </si>
+  <si>
+    <t>Haris KH</t>
   </si>
 </sst>
 </file>
@@ -420,6 +474,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -685,7 +743,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:Q59"/>
+  <dimension ref="A1:Q70"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="11.109375" customWidth="1"/>
@@ -2712,6 +2770,393 @@
         <v>22</v>
       </c>
     </row>
+    <row r="61" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A61">
+        <v>2533</v>
+      </c>
+      <c r="B61" s="1">
+        <v>45803</v>
+      </c>
+      <c r="C61">
+        <v>1033</v>
+      </c>
+      <c r="D61" t="s">
+        <v>114</v>
+      </c>
+      <c r="E61" t="s">
+        <v>115</v>
+      </c>
+      <c r="F61" t="s">
+        <v>17</v>
+      </c>
+      <c r="H61" t="s">
+        <v>18</v>
+      </c>
+      <c r="I61" s="1">
+        <v>42784</v>
+      </c>
+      <c r="J61" t="s">
+        <v>116</v>
+      </c>
+      <c r="K61">
+        <v>9633906039</v>
+      </c>
+      <c r="M61" t="s">
+        <v>20</v>
+      </c>
+      <c r="N61" t="s">
+        <v>117</v>
+      </c>
+      <c r="O61" t="s">
+        <v>17</v>
+      </c>
+      <c r="P61" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="62" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A62">
+        <v>2527</v>
+      </c>
+      <c r="B62" s="1">
+        <v>45798</v>
+      </c>
+      <c r="C62">
+        <v>1027</v>
+      </c>
+      <c r="D62" t="s">
+        <v>118</v>
+      </c>
+      <c r="E62" t="s">
+        <v>115</v>
+      </c>
+      <c r="F62" t="s">
+        <v>17</v>
+      </c>
+      <c r="H62" t="s">
+        <v>18</v>
+      </c>
+      <c r="I62" s="1">
+        <v>42830</v>
+      </c>
+      <c r="J62" t="s">
+        <v>93</v>
+      </c>
+      <c r="M62" t="s">
+        <v>20</v>
+      </c>
+      <c r="N62" t="s">
+        <v>117</v>
+      </c>
+      <c r="O62" t="s">
+        <v>17</v>
+      </c>
+      <c r="P62" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="63" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A63">
+        <v>2517</v>
+      </c>
+      <c r="B63" s="1">
+        <v>45796</v>
+      </c>
+      <c r="C63">
+        <v>1017</v>
+      </c>
+      <c r="D63" t="s">
+        <v>119</v>
+      </c>
+      <c r="E63" t="s">
+        <v>115</v>
+      </c>
+      <c r="F63" t="s">
+        <v>17</v>
+      </c>
+      <c r="H63" t="s">
+        <v>18</v>
+      </c>
+      <c r="I63" s="1">
+        <v>42809</v>
+      </c>
+      <c r="J63" t="s">
+        <v>120</v>
+      </c>
+      <c r="K63">
+        <v>971561091929</v>
+      </c>
+      <c r="M63" t="s">
+        <v>20</v>
+      </c>
+      <c r="N63" t="s">
+        <v>117</v>
+      </c>
+      <c r="O63" t="s">
+        <v>17</v>
+      </c>
+      <c r="P63" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="64" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A64">
+        <v>2515</v>
+      </c>
+      <c r="B64" s="1">
+        <v>45796</v>
+      </c>
+      <c r="C64">
+        <v>1015</v>
+      </c>
+      <c r="D64" t="s">
+        <v>121</v>
+      </c>
+      <c r="E64" t="s">
+        <v>115</v>
+      </c>
+      <c r="F64" t="s">
+        <v>17</v>
+      </c>
+      <c r="H64" t="s">
+        <v>27</v>
+      </c>
+      <c r="I64" s="1">
+        <v>42405</v>
+      </c>
+      <c r="J64" t="s">
+        <v>122</v>
+      </c>
+      <c r="K64">
+        <v>9061417328</v>
+      </c>
+      <c r="M64" t="s">
+        <v>20</v>
+      </c>
+      <c r="N64" t="s">
+        <v>117</v>
+      </c>
+      <c r="O64" t="s">
+        <v>17</v>
+      </c>
+      <c r="P64" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="65" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A65">
+        <v>2545</v>
+      </c>
+      <c r="B65" s="1">
+        <v>45807</v>
+      </c>
+      <c r="C65">
+        <v>1045</v>
+      </c>
+      <c r="D65" t="s">
+        <v>123</v>
+      </c>
+      <c r="E65" t="s">
+        <v>115</v>
+      </c>
+      <c r="F65" t="s">
+        <v>17</v>
+      </c>
+      <c r="H65" t="s">
+        <v>27</v>
+      </c>
+      <c r="I65" s="1">
+        <v>42528</v>
+      </c>
+      <c r="J65" t="s">
+        <v>124</v>
+      </c>
+      <c r="M65" t="s">
+        <v>20</v>
+      </c>
+      <c r="N65" t="s">
+        <v>117</v>
+      </c>
+      <c r="O65" t="s">
+        <v>17</v>
+      </c>
+      <c r="P65" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="66" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A66">
+        <v>2513</v>
+      </c>
+      <c r="B66" s="1">
+        <v>45796</v>
+      </c>
+      <c r="C66">
+        <v>1013</v>
+      </c>
+      <c r="D66" t="s">
+        <v>125</v>
+      </c>
+      <c r="E66" t="s">
+        <v>115</v>
+      </c>
+      <c r="F66" t="s">
+        <v>17</v>
+      </c>
+      <c r="H66" t="s">
+        <v>18</v>
+      </c>
+      <c r="I66" s="1">
+        <v>42647</v>
+      </c>
+      <c r="J66" t="s">
+        <v>100</v>
+      </c>
+      <c r="K66">
+        <v>8590691668</v>
+      </c>
+      <c r="M66" t="s">
+        <v>20</v>
+      </c>
+      <c r="N66" t="s">
+        <v>117</v>
+      </c>
+      <c r="O66" t="s">
+        <v>17</v>
+      </c>
+      <c r="P66" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="67" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A67">
+        <v>2566</v>
+      </c>
+      <c r="B67" s="1">
+        <v>45809</v>
+      </c>
+      <c r="C67">
+        <v>1066</v>
+      </c>
+      <c r="D67" t="s">
+        <v>126</v>
+      </c>
+      <c r="E67" t="s">
+        <v>115</v>
+      </c>
+      <c r="F67" t="s">
+        <v>17</v>
+      </c>
+      <c r="H67" t="s">
+        <v>18</v>
+      </c>
+      <c r="I67" s="1">
+        <v>42818</v>
+      </c>
+      <c r="J67" t="s">
+        <v>127</v>
+      </c>
+      <c r="M67" t="s">
+        <v>20</v>
+      </c>
+      <c r="N67" t="s">
+        <v>117</v>
+      </c>
+      <c r="O67" t="s">
+        <v>17</v>
+      </c>
+      <c r="P67" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="68" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A68">
+        <v>2519</v>
+      </c>
+      <c r="B68" s="1">
+        <v>45796</v>
+      </c>
+      <c r="C68">
+        <v>1019</v>
+      </c>
+      <c r="D68" t="s">
+        <v>128</v>
+      </c>
+      <c r="E68" t="s">
+        <v>115</v>
+      </c>
+      <c r="F68" t="s">
+        <v>17</v>
+      </c>
+      <c r="H68" t="s">
+        <v>27</v>
+      </c>
+      <c r="I68" s="1">
+        <v>42489</v>
+      </c>
+      <c r="J68" t="s">
+        <v>129</v>
+      </c>
+      <c r="K68">
+        <v>966502864767</v>
+      </c>
+      <c r="M68" t="s">
+        <v>20</v>
+      </c>
+      <c r="N68" t="s">
+        <v>117</v>
+      </c>
+      <c r="O68" t="s">
+        <v>17</v>
+      </c>
+      <c r="P68" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="70" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A70">
+        <v>2555</v>
+      </c>
+      <c r="B70" s="1">
+        <v>45796</v>
+      </c>
+      <c r="C70">
+        <v>1055</v>
+      </c>
+      <c r="D70" t="s">
+        <v>130</v>
+      </c>
+      <c r="E70" t="s">
+        <v>117</v>
+      </c>
+      <c r="F70" t="s">
+        <v>17</v>
+      </c>
+      <c r="H70" t="s">
+        <v>27</v>
+      </c>
+      <c r="I70" s="1">
+        <v>42808</v>
+      </c>
+      <c r="J70" t="s">
+        <v>131</v>
+      </c>
+      <c r="K70">
+        <v>9633311373</v>
+      </c>
+      <c r="M70" t="s">
+        <v>20</v>
+      </c>
+      <c r="N70" t="s">
+        <v>16</v>
+      </c>
+      <c r="O70" t="s">
+        <v>17</v>
+      </c>
+      <c r="P70" t="s">
+        <v>22</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>